<commit_message>
fix: Fix error when importing fnac products without images
</commit_message>
<xml_diff>
--- a/fnac/tests/test_models/test_inventory.xlsx
+++ b/fnac/tests/test_models/test_inventory.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1387" uniqueCount="329">
   <si>
     <t xml:space="preserve">RNG_SKU</t>
   </si>
@@ -972,9 +972,6 @@
   </si>
   <si>
     <t xml:space="preserve">627474176354</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14602133.jpg|33125883.jpg</t>
   </si>
   <si>
     <t xml:space="preserve">Green</t>
@@ -5838,9 +5835,7 @@
       <c r="Z30" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="AA30" s="1" t="s">
-        <v>305</v>
-      </c>
+      <c r="AA30" s="1"/>
       <c r="AB30" s="1" t="s">
         <v>297</v>
       </c>
@@ -5850,7 +5845,7 @@
       <c r="AF30" s="1"/>
       <c r="AG30" s="1"/>
       <c r="AH30" s="1" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AI30" s="1" t="s">
         <v>174</v>
@@ -5876,10 +5871,10 @@
         <v>85</v>
       </c>
       <c r="AX30" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="AY30" s="1" t="s">
         <v>307</v>
-      </c>
-      <c r="AY30" s="1" t="s">
-        <v>308</v>
       </c>
       <c r="AZ30" s="1" t="s">
         <v>301</v>
@@ -5936,7 +5931,7 @@
         <v>72</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H31" s="1" t="s">
         <v>290</v>
@@ -5945,7 +5940,7 @@
         <v>292</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>71</v>
@@ -5996,7 +5991,7 @@
         <v>71</v>
       </c>
       <c r="AA31" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="AB31" s="1" t="s">
         <v>297</v>
@@ -6007,7 +6002,7 @@
       <c r="AF31" s="1"/>
       <c r="AG31" s="1"/>
       <c r="AH31" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="AI31" s="1" t="s">
         <v>174</v>
@@ -6033,10 +6028,10 @@
         <v>85</v>
       </c>
       <c r="AX31" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="AY31" s="1" t="s">
         <v>313</v>
-      </c>
-      <c r="AY31" s="1" t="s">
-        <v>314</v>
       </c>
       <c r="AZ31" s="1" t="s">
         <v>301</v>
@@ -6077,10 +6072,10 @@
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>316</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>71</v>
@@ -6093,22 +6088,22 @@
         <v>72</v>
       </c>
       <c r="G32" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="H32" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="I32" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="I32" s="2" t="s">
+      <c r="J32" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="J32" s="1" t="s">
+      <c r="K32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="L32" s="1" t="s">
         <v>318</v>
-      </c>
-      <c r="K32" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="L32" s="1" t="s">
-        <v>319</v>
       </c>
       <c r="M32" s="1" t="s">
         <v>77</v>
@@ -6117,10 +6112,10 @@
         <v>71</v>
       </c>
       <c r="O32" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="P32" s="1" t="s">
         <v>320</v>
-      </c>
-      <c r="P32" s="1" t="s">
-        <v>321</v>
       </c>
       <c r="Q32" s="1" t="s">
         <v>71</v>
@@ -6153,10 +6148,10 @@
         <v>71</v>
       </c>
       <c r="AA32" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="AB32" s="1" t="s">
         <v>322</v>
-      </c>
-      <c r="AB32" s="1" t="s">
-        <v>323</v>
       </c>
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
@@ -6186,19 +6181,19 @@
         <v>85</v>
       </c>
       <c r="AX32" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="AY32" s="1" t="s">
         <v>324</v>
       </c>
-      <c r="AY32" s="1" t="s">
+      <c r="AZ32" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="AZ32" s="1" t="s">
+      <c r="BA32" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="BB32" s="1" t="s">
         <v>326</v>
-      </c>
-      <c r="BA32" s="1" t="s">
-        <v>320</v>
-      </c>
-      <c r="BB32" s="1" t="s">
-        <v>327</v>
       </c>
       <c r="BC32" s="1"/>
       <c r="BD32" s="1" t="s">
@@ -6220,10 +6215,10 @@
         <v>191</v>
       </c>
       <c r="BN32" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="BO32" s="1" t="s">
         <v>328</v>
-      </c>
-      <c r="BO32" s="1" t="s">
-        <v>329</v>
       </c>
       <c r="BP32" s="1"/>
       <c r="BQ32" s="1"/>

</xml_diff>

<commit_message>
fix: Fix fnac product import failing when description is empty
</commit_message>
<xml_diff>
--- a/fnac/tests/test_models/test_inventory.xlsx
+++ b/fnac/tests/test_models/test_inventory.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1387" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1386" uniqueCount="329">
   <si>
     <t xml:space="preserve">RNG_SKU</t>
   </si>
@@ -541,49 +541,49 @@
     <t xml:space="preserve">38M-DR0-NVN</t>
   </si>
   <si>
+    <t xml:space="preserve">8944099459733</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14603634.jpg|33125877.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J.085;JT.014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9D5-90B-A4A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J.085 - A625 - SSP - Adults Fleece Snood - One Size - BLACK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A625</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large Letter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PSW-84Z-6RR</t>
+  </si>
+  <si>
     <t xml:space="preserve">&lt;ul&gt;&lt;li&gt;Adjustable toggles allow to be tightened around the face.&lt;/li&gt;&lt;li&gt;Adults, one size fits all.&lt;/li&gt;&lt;li&gt;Made from 100% Polyester.&lt;/li&gt;&lt;/ul&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8944099459733</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.99</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14603634.jpg|33125877.jpg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J.085;JT.014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Black</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One Size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9D5-90B-A4A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J.085 - A625 - SSP - Adults Fleece Snood - One Size - BLACK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A625</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Large Letter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PSW-84Z-6RR</t>
   </si>
   <si>
     <t xml:space="preserve">8944099459719</t>
@@ -3114,17 +3114,15 @@
       <c r="H13" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="I13" s="1"/>
+      <c r="J13" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="K13" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="1" t="s">
         <v>168</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>169</v>
       </c>
       <c r="M13" s="1" t="s">
         <v>77</v>
@@ -3136,7 +3134,7 @@
         <v>155</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q13" s="1" t="s">
         <v>71</v>
@@ -3169,10 +3167,10 @@
         <v>71</v>
       </c>
       <c r="AA13" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB13" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="AB13" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="AC13" s="1"/>
       <c r="AD13" s="1"/>
@@ -3180,10 +3178,10 @@
       <c r="AF13" s="1"/>
       <c r="AG13" s="1"/>
       <c r="AH13" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="AI13" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="AI13" s="1" t="s">
-        <v>174</v>
       </c>
       <c r="AJ13" s="1"/>
       <c r="AK13" s="1"/>
@@ -3206,19 +3204,19 @@
         <v>85</v>
       </c>
       <c r="AX13" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="AY13" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="AY13" s="1" t="s">
+      <c r="AZ13" s="1" t="s">
         <v>176</v>
-      </c>
-      <c r="AZ13" s="1" t="s">
-        <v>177</v>
       </c>
       <c r="BA13" s="1" t="s">
         <v>155</v>
       </c>
       <c r="BB13" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="BC13" s="1"/>
       <c r="BD13" s="1" t="s">
@@ -3230,7 +3228,7 @@
       </c>
       <c r="BG13" s="1"/>
       <c r="BH13" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI13" s="1"/>
       <c r="BJ13" s="1"/>
@@ -3266,13 +3264,13 @@
         <v>72</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>164</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>181</v>
@@ -3281,7 +3279,7 @@
         <v>182</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="M14" s="1" t="s">
         <v>77</v>
@@ -3340,7 +3338,7 @@
         <v>186</v>
       </c>
       <c r="AI14" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ14" s="1"/>
       <c r="AK14" s="1"/>
@@ -3369,13 +3367,13 @@
         <v>188</v>
       </c>
       <c r="AZ14" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="BA14" s="1" t="s">
         <v>155</v>
       </c>
       <c r="BB14" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="BC14" s="1"/>
       <c r="BD14" s="1" t="s">
@@ -3387,7 +3385,7 @@
       </c>
       <c r="BG14" s="1"/>
       <c r="BH14" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI14" s="1"/>
       <c r="BJ14" s="1"/>
@@ -3429,7 +3427,7 @@
         <v>164</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>190</v>
@@ -3438,7 +3436,7 @@
         <v>191</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="M15" s="1" t="s">
         <v>77</v>
@@ -3497,7 +3495,7 @@
         <v>194</v>
       </c>
       <c r="AI15" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ15" s="1"/>
       <c r="AK15" s="1"/>
@@ -3526,13 +3524,13 @@
         <v>196</v>
       </c>
       <c r="AZ15" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="BA15" s="1" t="s">
         <v>155</v>
       </c>
       <c r="BB15" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="BC15" s="1"/>
       <c r="BD15" s="1" t="s">
@@ -3544,7 +3542,7 @@
       </c>
       <c r="BG15" s="1"/>
       <c r="BH15" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI15" s="1"/>
       <c r="BJ15" s="1"/>
@@ -3607,7 +3605,7 @@
         <v>155</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q16" s="1" t="s">
         <v>71</v>
@@ -3699,7 +3697,7 @@
       </c>
       <c r="BG16" s="1"/>
       <c r="BH16" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI16" s="1"/>
       <c r="BJ16" s="1"/>
@@ -3856,7 +3854,7 @@
       </c>
       <c r="BG17" s="1"/>
       <c r="BH17" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI17" s="1"/>
       <c r="BJ17" s="1"/>
@@ -4013,7 +4011,7 @@
       </c>
       <c r="BG18" s="1"/>
       <c r="BH18" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI18" s="1"/>
       <c r="BJ18" s="1"/>
@@ -4170,7 +4168,7 @@
       </c>
       <c r="BG19" s="1"/>
       <c r="BH19" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI19" s="1"/>
       <c r="BJ19" s="1"/>
@@ -4327,7 +4325,7 @@
       </c>
       <c r="BG20" s="1"/>
       <c r="BH20" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI20" s="1"/>
       <c r="BJ20" s="1"/>
@@ -4434,7 +4432,7 @@
       <c r="AF21" s="1"/>
       <c r="AG21" s="1"/>
       <c r="AH21" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AI21" s="1" t="s">
         <v>220</v>
@@ -4484,7 +4482,7 @@
       </c>
       <c r="BG21" s="1"/>
       <c r="BH21" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI21" s="1"/>
       <c r="BJ21" s="1"/>
@@ -4591,7 +4589,7 @@
       <c r="AF22" s="1"/>
       <c r="AG22" s="1"/>
       <c r="AH22" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AI22" s="1" t="s">
         <v>228</v>
@@ -4641,7 +4639,7 @@
       </c>
       <c r="BG22" s="1"/>
       <c r="BH22" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI22" s="1"/>
       <c r="BJ22" s="1"/>
@@ -4748,7 +4746,7 @@
       <c r="AF23" s="1"/>
       <c r="AG23" s="1"/>
       <c r="AH23" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AI23" s="1" t="s">
         <v>235</v>
@@ -4798,7 +4796,7 @@
       </c>
       <c r="BG23" s="1"/>
       <c r="BH23" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI23" s="1"/>
       <c r="BJ23" s="1"/>
@@ -4905,7 +4903,7 @@
       <c r="AF24" s="1"/>
       <c r="AG24" s="1"/>
       <c r="AH24" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AI24" s="1" t="s">
         <v>241</v>
@@ -4955,7 +4953,7 @@
       </c>
       <c r="BG24" s="1"/>
       <c r="BH24" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI24" s="1"/>
       <c r="BJ24" s="1"/>
@@ -5112,7 +5110,7 @@
       </c>
       <c r="BG25" s="1"/>
       <c r="BH25" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI25" s="1"/>
       <c r="BJ25" s="1"/>
@@ -5269,7 +5267,7 @@
       </c>
       <c r="BG26" s="1"/>
       <c r="BH26" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI26" s="1"/>
       <c r="BJ26" s="1"/>
@@ -5426,7 +5424,7 @@
       </c>
       <c r="BG27" s="1"/>
       <c r="BH27" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI27" s="1"/>
       <c r="BJ27" s="1"/>
@@ -5583,7 +5581,7 @@
       </c>
       <c r="BG28" s="1"/>
       <c r="BH28" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI28" s="1"/>
       <c r="BJ28" s="1"/>
@@ -5693,7 +5691,7 @@
         <v>298</v>
       </c>
       <c r="AI29" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ29" s="1"/>
       <c r="AK29" s="1"/>
@@ -5740,7 +5738,7 @@
       </c>
       <c r="BG29" s="1"/>
       <c r="BH29" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI29" s="1"/>
       <c r="BJ29" s="1"/>
@@ -5803,7 +5801,7 @@
         <v>295</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Q30" s="1" t="s">
         <v>71</v>
@@ -5848,7 +5846,7 @@
         <v>305</v>
       </c>
       <c r="AI30" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ30" s="1"/>
       <c r="AK30" s="1"/>
@@ -5895,7 +5893,7 @@
       </c>
       <c r="BG30" s="1"/>
       <c r="BH30" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI30" s="1"/>
       <c r="BJ30" s="1"/>
@@ -6005,7 +6003,7 @@
         <v>311</v>
       </c>
       <c r="AI31" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AJ31" s="1"/>
       <c r="AK31" s="1"/>
@@ -6052,7 +6050,7 @@
       </c>
       <c r="BG31" s="1"/>
       <c r="BH31" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI31" s="1"/>
       <c r="BJ31" s="1"/>
@@ -6205,7 +6203,7 @@
       </c>
       <c r="BG32" s="1"/>
       <c r="BH32" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BI32" s="1"/>
       <c r="BJ32" s="1"/>

</xml_diff>